<commit_message>
Fix report-checklist.xlsx per feedback Sogei
- C011: Fix colonna K (RAZIONALE DI APPLICABILITA') per casi N/A -
  correzione maiuscola iniziale e apostrofo Unicode U+2019
- C007: Aggiunta colonne Q (coda retry) e R (invio manuale) per
  casi KO applicabili 156, 169, 468
- C010: Aggiunta colonna H (traceId) per casi OK 448, 449 -
  ri-eseguiti test per catturare traceId dalla response
- Aggiornati data.json e PDF per casi 448, 449 con nuovi risultati
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111#MEDILUSTSRLXX/Medilust_Srl/Mami/1.0.0/report-checklist.xlsx
+++ b/GATEWAY/A1#111#MEDILUSTSRLXX/Medilust_Srl/Mami/1.0.0/report-checklist.xlsx
@@ -2988,8 +2988,16 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="Q15" s="32" t="n"/>
-      <c r="R15" s="32" t="n"/>
+      <c r="Q15" s="32" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="R15" s="32" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
       <c r="S15" s="32" t="inlineStr">
         <is>
           <t>L'errore viene visualizzato al medico che puo' correggere il documento e riprovare l'invio al FSE. Il medico puo' proseguire con il processo clinico indipendentemente dall'esito dell'invio.</t>
@@ -3432,8 +3440,16 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="Q23" s="32" t="n"/>
-      <c r="R23" s="32" t="n"/>
+      <c r="Q23" s="32" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="R23" s="32" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
       <c r="S23" s="32" t="inlineStr">
         <is>
           <t>L'errore viene visualizzato al medico che puo' correggere il documento e riprovare l'invio al FSE. Il medico puo' proseguire con il processo clinico indipendentemente dall'esito dell'invio.</t>
@@ -8005,8 +8021,16 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="Q116" s="32" t="n"/>
-      <c r="R116" s="32" t="n"/>
+      <c r="Q116" s="32" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="R116" s="32" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
       <c r="S116" s="32" t="inlineStr">
         <is>
           <t>L'errore viene visualizzato al medico che puo' correggere il documento e riprovare l'invio al FSE. Il medico puo' proseguire con il processo clinico indipendentemente dall'esito dell'invio.</t>
@@ -8093,8 +8117,16 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="Q117" s="32" t="n"/>
-      <c r="R117" s="32" t="n"/>
+      <c r="Q117" s="32" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="R117" s="32" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
       <c r="S117" s="32" t="inlineStr">
         <is>
           <t>L'errore viene visualizzato al medico che puo' correggere il documento e riprovare l'invio al FSE. Il medico puo' proseguire con il processo clinico indipendentemente dall'esito dell'invio.</t>
@@ -8181,8 +8213,16 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="Q118" s="32" t="n"/>
-      <c r="R118" s="32" t="n"/>
+      <c r="Q118" s="32" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="R118" s="32" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
       <c r="S118" s="32" t="inlineStr">
         <is>
           <t>L'errore viene visualizzato al medico che puo' correggere il documento e riprovare l'invio al FSE. Il medico puo' proseguire con il processo clinico indipendentemente dall'esito dell'invio.</t>
@@ -8265,8 +8305,16 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="Q119" s="32" t="n"/>
-      <c r="R119" s="32" t="n"/>
+      <c r="Q119" s="32" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="R119" s="32" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
       <c r="S119" s="32" t="inlineStr">
         <is>
           <t>L'errore viene visualizzato al medico che puo' correggere il documento e riprovare l'invio al FSE. Il medico puo' proseguire con il processo clinico indipendentemente dall'esito dell'invio.</t>
@@ -8317,7 +8365,7 @@
       </c>
       <c r="K120" s="32" t="inlineStr">
         <is>
-          <t>campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
+          <t>Campo/sezione non gestito/a in modo strutturato dall’applicativo</t>
         </is>
       </c>
       <c r="L120" s="32" t="n"/>
@@ -8409,8 +8457,16 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="Q121" s="32" t="n"/>
-      <c r="R121" s="32" t="n"/>
+      <c r="Q121" s="32" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="R121" s="32" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
       <c r="S121" s="32" t="inlineStr">
         <is>
           <t>L'errore viene visualizzato al medico che puo' correggere il documento e riprovare l'invio al FSE. Il medico puo' proseguire con il processo clinico indipendentemente dall'esito dell'invio.</t>
@@ -8497,8 +8553,16 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="Q122" s="32" t="n"/>
-      <c r="R122" s="32" t="n"/>
+      <c r="Q122" s="32" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="R122" s="32" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
       <c r="S122" s="32" t="inlineStr">
         <is>
           <t>L'errore viene visualizzato al medico che puo' correggere il documento e riprovare l'invio al FSE. Il medico puo' proseguire con il processo clinico indipendentemente dall'esito dell'invio.</t>
@@ -8549,7 +8613,7 @@
       </c>
       <c r="K123" s="32" t="inlineStr">
         <is>
-          <t>campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
+          <t>Campo/sezione non gestito/a in modo strutturato dall’applicativo</t>
         </is>
       </c>
       <c r="L123" s="32" t="n"/>
@@ -8641,8 +8705,16 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="Q124" s="32" t="n"/>
-      <c r="R124" s="32" t="n"/>
+      <c r="Q124" s="32" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="R124" s="32" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
       <c r="S124" s="32" t="inlineStr">
         <is>
           <t>L'errore viene visualizzato al medico che puo' correggere il documento e riprovare l'invio al FSE. Il medico puo' proseguire con il processo clinico indipendentemente dall'esito dell'invio.</t>
@@ -8693,7 +8765,7 @@
       </c>
       <c r="K125" s="32" t="inlineStr">
         <is>
-          <t>campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
+          <t>Campo/sezione non gestito/a in modo strutturato dall’applicativo</t>
         </is>
       </c>
       <c r="L125" s="32" t="n"/>
@@ -8749,7 +8821,7 @@
       </c>
       <c r="K126" s="32" t="inlineStr">
         <is>
-          <t>campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
+          <t>Campo/sezione non gestito/a in modo strutturato dall’applicativo</t>
         </is>
       </c>
       <c r="L126" s="32" t="n"/>
@@ -8805,7 +8877,7 @@
       </c>
       <c r="K127" s="32" t="inlineStr">
         <is>
-          <t>campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
+          <t>Campo/sezione non gestito/a in modo strutturato dall’applicativo</t>
         </is>
       </c>
       <c r="L127" s="32" t="n"/>
@@ -8861,7 +8933,7 @@
       </c>
       <c r="K128" s="32" t="inlineStr">
         <is>
-          <t>campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
+          <t>Campo/sezione non gestito/a in modo strutturato dall’applicativo</t>
         </is>
       </c>
       <c r="L128" s="32" t="n"/>
@@ -8917,7 +8989,7 @@
       </c>
       <c r="K129" s="32" t="inlineStr">
         <is>
-          <t>l'applicativo effettua controlli preventivi sul dato inserito</t>
+          <t>L’applicativo effettua controlli preventivi sul dato inserito</t>
         </is>
       </c>
       <c r="L129" s="32" t="n"/>
@@ -9005,8 +9077,16 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="Q130" s="32" t="n"/>
-      <c r="R130" s="32" t="n"/>
+      <c r="Q130" s="32" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="R130" s="32" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
       <c r="S130" s="32" t="inlineStr">
         <is>
           <t>L'errore viene visualizzato al medico che puo' correggere il documento e riprovare l'invio al FSE. Il medico puo' proseguire con il processo clinico indipendentemente dall'esito dell'invio.</t>
@@ -10654,10 +10734,14 @@
           <t>2026-03-26T09:30:00Z</t>
         </is>
       </c>
-      <c r="H164" s="31" t="inlineStr"/>
+      <c r="H164" s="31" t="inlineStr">
+        <is>
+          <t>67d351a5998a034a68757430bfcbf8a9</t>
+        </is>
+      </c>
       <c r="I164" s="36" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.b7105f44e4e877d8218cdbd9e1f9d3e52ad7f095830f157702c31ba8bf910704.5cd615d671^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.c443f556077c72dde4f063dc5f068b0fb667f0bc00f9ecefd88d57b2d1381cad.9dd27abb86^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J164" s="32" t="inlineStr">
@@ -10718,10 +10802,14 @@
           <t>2026-03-26T09:30:00Z</t>
         </is>
       </c>
-      <c r="H165" s="31" t="inlineStr"/>
+      <c r="H165" s="31" t="inlineStr">
+        <is>
+          <t>c49ec8daa487cedb2caf3083eff4ac79</t>
+        </is>
+      </c>
       <c r="I165" s="36" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.2282334ada07019de1b1eebc8e9be4a619b3c78ad2fcb2819b3af594adbe7382.bb41df4bce^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.cff74446fb87f52b1f0d441f5e7ea36b0ab25efb2b5722318956c3fd9c292725.dc5609a0e4^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J165" s="32" t="inlineStr">
@@ -11264,7 +11352,7 @@
       </c>
       <c r="K176" s="32" t="inlineStr">
         <is>
-          <t>campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
+          <t>Campo/sezione non gestito/a in modo strutturato dall’applicativo</t>
         </is>
       </c>
       <c r="L176" s="29" t="n"/>
@@ -11640,8 +11728,16 @@
           <t>NO</t>
         </is>
       </c>
-      <c r="Q183" s="32" t="n"/>
-      <c r="R183" s="32" t="n"/>
+      <c r="Q183" s="32" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="R183" s="32" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
       <c r="S183" s="29" t="inlineStr">
         <is>
           <t>L'errore viene visualizzato al medico che puo' correggere il documento e riprovare l'invio al FSE. Il medico puo' proseguire con il processo clinico indipendentemente dall'esito dell'invio.</t>
@@ -11980,7 +12076,7 @@
       </c>
       <c r="K190" s="32" t="inlineStr">
         <is>
-          <t>campo/sezione non gestito/a in modo strutturato dall'applicativo</t>
+          <t>Campo/sezione non gestito/a in modo strutturato dall’applicativo</t>
         </is>
       </c>
       <c r="L190" s="32" t="n"/>

</xml_diff>

<commit_message>
Fix report-checklist per feedback Sogei
- Header: spostati NOME FORNITORE e subject_application_* in colonna C/D
- C007: valorizzate colonne I (workflowInstanceId), Q (retry), R (invio manuale)
  per tutti i casi KO applicabili
- C011: corretti valori colonna K con dropdown esatto del template V9.0.0
- C010: aggiunto traceId (col H) per casi OK 448, 449
- Ri-eseguiti test 32, 40, 156, 169, 448, 449, 468 per catturare
  traceId e workflowInstanceId dalle risposte del Gateway
- Aggiornati data.json e PDF con i nuovi risultati
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111#MEDILUSTSRLXX/Medilust_Srl/Mami/1.0.0/report-checklist.xlsx
+++ b/GATEWAY/A1#111#MEDILUSTSRLXX/Medilust_Srl/Mami/1.0.0/report-checklist.xlsx
@@ -2353,13 +2353,12 @@
         </is>
       </c>
       <c r="B2" s="82" t="n"/>
-      <c r="C2" s="83" t="n"/>
+      <c r="C2" s="83" t="inlineStr">
+        <is>
+          <t>Medilust Srl</t>
+        </is>
+      </c>
       <c r="D2" s="82" t="n"/>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Medilust Srl</t>
-        </is>
-      </c>
       <c r="F2" s="6" t="n"/>
       <c r="G2" s="6" t="n"/>
       <c r="H2" s="6" t="n"/>
@@ -2388,15 +2387,10 @@
       <c r="B3" s="84" t="n"/>
       <c r="C3" s="85" t="inlineStr">
         <is>
-          <t>subject_application_id:</t>
+          <t>subject_application_id: Mami</t>
         </is>
       </c>
       <c r="D3" s="82" t="n"/>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Mami</t>
-        </is>
-      </c>
       <c r="F3" s="6" t="n"/>
       <c r="G3" s="6" t="n"/>
       <c r="H3" s="6" t="n"/>
@@ -2421,15 +2415,11 @@
       <c r="B4" s="87" t="n"/>
       <c r="C4" s="85" t="inlineStr">
         <is>
-          <t>subject_application_vendor:</t>
+          <t>subject_application_vendor: Medilust Srl</t>
         </is>
       </c>
       <c r="D4" s="82" t="n"/>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>Medilust Srl</t>
-        </is>
-      </c>
+      <c r="E4" s="4" t="n"/>
       <c r="F4" s="6" t="n"/>
       <c r="G4" s="6" t="n"/>
       <c r="H4" s="6" t="n"/>
@@ -2454,15 +2444,10 @@
       <c r="B5" s="89" t="n"/>
       <c r="C5" s="85" t="inlineStr">
         <is>
-          <t>subject_application_version:</t>
+          <t>subject_application_version: 1.0.0</t>
         </is>
       </c>
       <c r="D5" s="82" t="n"/>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>1.0.0</t>
-        </is>
-      </c>
       <c r="F5" s="6" t="n"/>
       <c r="G5" s="6" t="n"/>
       <c r="H5" s="6" t="n"/>
@@ -2957,10 +2942,14 @@
       </c>
       <c r="H15" s="31" t="inlineStr">
         <is>
-          <t>fb5aa5f1216bda7423db3ddd3fa4f167</t>
-        </is>
-      </c>
-      <c r="I15" s="36" t="inlineStr"/>
+          <t>024395bb00a2d73104acb2ef1119190d</t>
+        </is>
+      </c>
+      <c r="I15" s="36" t="inlineStr">
+        <is>
+          <t>UNKNOWN_WORKFLOW_ID</t>
+        </is>
+      </c>
       <c r="J15" s="32" t="inlineStr">
         <is>
           <t>SI</t>
@@ -3409,10 +3398,14 @@
       </c>
       <c r="H23" s="31" t="inlineStr">
         <is>
-          <t>6be906828c7b97163a3cb2255113efe9</t>
-        </is>
-      </c>
-      <c r="I23" s="36" t="inlineStr"/>
+          <t>028d8c894db8b48550ef3d6a433001c7</t>
+        </is>
+      </c>
+      <c r="I23" s="36" t="inlineStr">
+        <is>
+          <t>UNKNOWN_WORKFLOW_ID</t>
+        </is>
+      </c>
       <c r="J23" s="32" t="inlineStr">
         <is>
           <t>SI</t>
@@ -3886,7 +3879,11 @@
           <t>SI</t>
         </is>
       </c>
-      <c r="R31" s="32" t="n"/>
+      <c r="R31" s="32" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
       <c r="S31" s="32" t="inlineStr">
         <is>
           <t>L'applicativo implementa una coda di retry automatica (Oban job queue) che ripete l'invio del documento fino a 5 tentativi con backoff esponenziale. L'errore viene segnalato al medico che puo' monitorare lo stato dell'invio dalla dashboard.</t>
@@ -8274,10 +8271,14 @@
       </c>
       <c r="H119" s="31" t="inlineStr">
         <is>
-          <t>91e2978518604ddc196b812c5a5325a1</t>
-        </is>
-      </c>
-      <c r="I119" s="36" t="inlineStr"/>
+          <t>029a2687488ea0e628139f7d148dd19b</t>
+        </is>
+      </c>
+      <c r="I119" s="36" t="inlineStr">
+        <is>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.720eeebcb3efeab65ab10056d3d99f133ee02fb902179d4940474eff955ffc06.7cf6f4d19e^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+        </is>
+      </c>
       <c r="J119" s="32" t="inlineStr">
         <is>
           <t>SI</t>
@@ -9046,10 +9047,14 @@
       </c>
       <c r="H130" s="31" t="inlineStr">
         <is>
-          <t>92e7c764fe8aea940971f80b79bc0aa9</t>
-        </is>
-      </c>
-      <c r="I130" s="36" t="inlineStr"/>
+          <t>3b6f321798d6c8281ca6f03d8c811596</t>
+        </is>
+      </c>
+      <c r="I130" s="36" t="inlineStr">
+        <is>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.a5ebda750cd8c99dddf1784474845ba01e47c77ce720a201a2e8a5d51cc35d02.e05041c657^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+        </is>
+      </c>
       <c r="J130" s="32" t="inlineStr">
         <is>
           <t>SI</t>
@@ -11697,10 +11702,14 @@
       </c>
       <c r="H183" s="29" t="inlineStr">
         <is>
-          <t>9469f9f6e80e95e2d34a92a9deb27e9c</t>
-        </is>
-      </c>
-      <c r="I183" s="29" t="inlineStr"/>
+          <t>51aeac34e4273ad5bb4a048cf6761cbf</t>
+        </is>
+      </c>
+      <c r="I183" s="29" t="inlineStr">
+        <is>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.83b7facea951fbf9cf2aa774efd537186daca1353da32edb0cb4f1d2832bed58.3bfeee1273^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+        </is>
+      </c>
       <c r="J183" s="32" t="inlineStr">
         <is>
           <t>SI</t>

</xml_diff>

<commit_message>
Fix test cases 448, 449 per medilust_srl/mami/1.0.0
Ri-eseguiti tutti i test case RSA con CDA allineato ai documenti
di riferimento CT24/CT25.

Risultati: 2 OK + 11 KO + 10 N/A + 1 timeout
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111#MEDILUSTSRLXX/Medilust_Srl/Mami/1.0.0/report-checklist.xlsx
+++ b/GATEWAY/A1#111#MEDILUSTSRLXX/Medilust_Srl/Mami/1.0.0/report-checklist.xlsx
@@ -2932,17 +2932,17 @@
       </c>
       <c r="F15" s="31" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="G15" s="31" t="inlineStr">
         <is>
-          <t>2026-03-26T09:30:00Z</t>
+          <t>2026-03-30T10:18:56.373142Z</t>
         </is>
       </c>
       <c r="H15" s="31" t="inlineStr">
         <is>
-          <t>024395bb00a2d73104acb2ef1119190d</t>
+          <t>e341915c6d3e1f472d97cdcb971fb5a2</t>
         </is>
       </c>
       <c r="I15" s="36" t="inlineStr">
@@ -3388,17 +3388,17 @@
       </c>
       <c r="F23" s="31" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="G23" s="31" t="inlineStr">
         <is>
-          <t>2026-03-26T09:30:00Z</t>
+          <t>2026-03-30T10:18:56.373144Z</t>
         </is>
       </c>
       <c r="H23" s="31" t="inlineStr">
         <is>
-          <t>028d8c894db8b48550ef3d6a433001c7</t>
+          <t>758af7b4f290de78f71ef2edaca93bed</t>
         </is>
       </c>
       <c r="I23" s="36" t="inlineStr">
@@ -7973,22 +7973,22 @@
       </c>
       <c r="F116" s="31" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="G116" s="31" t="inlineStr">
         <is>
-          <t>2026-03-26T09:30:00Z</t>
+          <t>2026-03-30T10:18:56.373146Z</t>
         </is>
       </c>
       <c r="H116" s="31" t="inlineStr">
         <is>
-          <t>fd53aefe28e293c42c9b461b72f1ce4e</t>
+          <t>97be6698fb0ab4b731c208d1619ce938</t>
         </is>
       </c>
       <c r="I116" s="36" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.dd71a78aab8b523897d764c75a06f8efa0fba722885e891dea7e0baf93bc76a7.22a27f218d^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.331939b21588d65462217c807dfe9db215db18fd1bee3182c0582922187c37af.5cc0a65362^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J116" s="32" t="inlineStr">
@@ -8069,22 +8069,22 @@
       </c>
       <c r="F117" s="31" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="G117" s="31" t="inlineStr">
         <is>
-          <t>2026-03-26T09:30:00Z</t>
+          <t>2026-03-30T10:18:56.373148Z</t>
         </is>
       </c>
       <c r="H117" s="31" t="inlineStr">
         <is>
-          <t>7327b09b747581f4ddb9ac24401b0aaf</t>
+          <t>9b20623b5aa59e39557174ec4bb95dff</t>
         </is>
       </c>
       <c r="I117" s="36" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.58a48b3463aa6c5cc61c5ea32103c81afadc6910686c8c11dbdebccc1b7c6fa4.a6ffefe97c^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.11c6b0631b8cffdbe0c4dd5103ab1f3d0964fbcdd7c603d3d723f0cc0c0e9022.91e8aaf702^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J117" s="32" t="inlineStr">
@@ -8165,22 +8165,22 @@
       </c>
       <c r="F118" s="31" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="G118" s="31" t="inlineStr">
         <is>
-          <t>2026-03-26T09:30:00Z</t>
+          <t>2026-03-30T10:18:56.373149Z</t>
         </is>
       </c>
       <c r="H118" s="31" t="inlineStr">
         <is>
-          <t>739f76945087663307e3cb56630272a8</t>
+          <t>116178cc142dba50b6187bac9116c45d</t>
         </is>
       </c>
       <c r="I118" s="36" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.9b8bf733f34c910993d6d51ee93f509fba285fcab950951a28bd399101ec3ac8.d26d09ff38^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.cdc96161f479cbfa78953c74a2f82337d728fd81c8bd8b56031d7b5fb490cc12.8f6f5a8e55^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J118" s="32" t="inlineStr">
@@ -8261,22 +8261,22 @@
       </c>
       <c r="F119" s="31" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="G119" s="31" t="inlineStr">
         <is>
-          <t>2026-03-26T09:30:00Z</t>
+          <t>2026-03-30T10:18:56.373177Z</t>
         </is>
       </c>
       <c r="H119" s="31" t="inlineStr">
         <is>
-          <t>029a2687488ea0e628139f7d148dd19b</t>
+          <t>fe4f7521a2952d9f29324cc05b356501</t>
         </is>
       </c>
       <c r="I119" s="36" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.720eeebcb3efeab65ab10056d3d99f133ee02fb902179d4940474eff955ffc06.7cf6f4d19e^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.1297897c909cfa42597c8da00d9624f362ab88b022d6a5fb9cd035204403a5f3.8802b8b879^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J119" s="32" t="inlineStr">
@@ -8413,22 +8413,22 @@
       </c>
       <c r="F121" s="31" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="G121" s="31" t="inlineStr">
         <is>
-          <t>2026-03-26T09:30:00Z</t>
+          <t>2026-03-30T10:18:56.373179Z</t>
         </is>
       </c>
       <c r="H121" s="31" t="inlineStr">
         <is>
-          <t>fb64e4753c47fafbc6d35375448244a8</t>
+          <t>23a84357d775dff55faffa09a2c3a8c1</t>
         </is>
       </c>
       <c r="I121" s="36" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.7efb794767eaa1d1c412c1d9d22803a02bcb3e83e0c72efb4095e0198d9ca6b0.ec0b9f9582^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.71e65b5a57b9a5a687feeb43a6d8453b4f6873e7f0ecb88ba80056f9662cdec7.10080fc657^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J121" s="32" t="inlineStr">
@@ -8509,22 +8509,22 @@
       </c>
       <c r="F122" s="31" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="G122" s="31" t="inlineStr">
         <is>
-          <t>2026-03-26T09:30:00Z</t>
+          <t>2026-03-30T10:18:56.373181Z</t>
         </is>
       </c>
       <c r="H122" s="31" t="inlineStr">
         <is>
-          <t>ba39f6fb4a58ae380274234a67c5de29</t>
+          <t>b3ce02f5258c0fb07e69fba2308ae8ef</t>
         </is>
       </c>
       <c r="I122" s="36" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.0eedf6a98de7632236de5589093a7036cdf4dd4892c3d98e9268265921ca9b29.a515e4acd3^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.3ab867b2426a85d90cc1abb1ee4408c0ee918497ed6ef337eac621bd7a161ba0.e1020f6630^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J122" s="32" t="inlineStr">
@@ -8661,22 +8661,22 @@
       </c>
       <c r="F124" s="31" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="G124" s="31" t="inlineStr">
         <is>
-          <t>2026-03-26T09:30:00Z</t>
+          <t>2026-03-30T10:18:56.373183Z</t>
         </is>
       </c>
       <c r="H124" s="31" t="inlineStr">
         <is>
-          <t>408e08e88c1ffde6d77674372039f190</t>
+          <t>c9bd14a0ff9b7cce8e420c35b029ab58</t>
         </is>
       </c>
       <c r="I124" s="36" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.f1fe511dd46bdbb186fd259f02530abcde477991b02b3237e32f922fb8e75ab9.0e84c68fde^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.5038033db023b45100e24712fa5fe39719c64c2479ffb28b8276ec299bea83df.7c159f6684^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J124" s="32" t="inlineStr">
@@ -9037,22 +9037,22 @@
       </c>
       <c r="F130" s="31" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="G130" s="31" t="inlineStr">
         <is>
-          <t>2026-03-26T09:30:00Z</t>
+          <t>2026-03-30T10:18:56.373184Z</t>
         </is>
       </c>
       <c r="H130" s="31" t="inlineStr">
         <is>
-          <t>3b6f321798d6c8281ca6f03d8c811596</t>
+          <t>320a998aa085823859222a2259b4b77c</t>
         </is>
       </c>
       <c r="I130" s="36" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.a5ebda750cd8c99dddf1784474845ba01e47c77ce720a201a2e8a5d51cc35d02.e05041c657^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.9d8d599dbab4551922a7ec336437cd8ecf96f436900ba77e4ef6e2df3c65ec42.925f211a3d^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J130" s="32" t="inlineStr">
@@ -10731,22 +10731,22 @@
       </c>
       <c r="F164" s="31" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="G164" s="31" t="inlineStr">
         <is>
-          <t>2026-03-26T09:30:00Z</t>
+          <t>2026-03-30T10:18:56.373085Z</t>
         </is>
       </c>
       <c r="H164" s="31" t="inlineStr">
         <is>
-          <t>67d351a5998a034a68757430bfcbf8a9</t>
+          <t>59dc7268b603f5006cb23c0378f5eed5</t>
         </is>
       </c>
       <c r="I164" s="36" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.c443f556077c72dde4f063dc5f068b0fb667f0bc00f9ecefd88d57b2d1381cad.9dd27abb86^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.0dd4f3a86924a9544353276f9c0ecc9f445c9734bdbade991fcad6ecd2a60bd1.2017f9aa77^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J164" s="32" t="inlineStr">
@@ -10799,22 +10799,22 @@
       </c>
       <c r="F165" s="31" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="G165" s="31" t="inlineStr">
         <is>
-          <t>2026-03-26T09:30:00Z</t>
+          <t>2026-03-30T10:18:56.373139Z</t>
         </is>
       </c>
       <c r="H165" s="31" t="inlineStr">
         <is>
-          <t>c49ec8daa487cedb2caf3083eff4ac79</t>
+          <t>f8396c60246beea23fae8f43329dae1d</t>
         </is>
       </c>
       <c r="I165" s="36" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.cff74446fb87f52b1f0d441f5e7ea36b0ab25efb2b5722318956c3fd9c292725.dc5609a0e4^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.f813144e0cd96b8b6652e522b89c2a5ff9c4798c6395231cce22008ea2fc958f.ca6285e102^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J165" s="32" t="inlineStr">
@@ -11692,22 +11692,22 @@
       </c>
       <c r="F183" s="29" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-30</t>
         </is>
       </c>
       <c r="G183" s="29" t="inlineStr">
         <is>
-          <t>2026-03-26T09:30:00Z</t>
+          <t>2026-03-30T10:18:56.373186Z</t>
         </is>
       </c>
       <c r="H183" s="29" t="inlineStr">
         <is>
-          <t>51aeac34e4273ad5bb4a048cf6761cbf</t>
+          <t>30809de819f2718028776d2f225576f3</t>
         </is>
       </c>
       <c r="I183" s="29" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.83b7facea951fbf9cf2aa774efd537186daca1353da32edb0cb4f1d2832bed58.3bfeee1273^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.5c9418f0aee8bfae73f29e4db028b29cdca87ac640dc005a3e47fae91a89ef1c.731f7692ac^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J183" s="32" t="inlineStr">

</xml_diff>

<commit_message>
Fix test cases 448, 449 (CT24/CT25) per medilust_srl/mami/1.0.0
CDA allineato ai documenti di riferimento CT24 e CT25:
- Corretti displayName sezioni (Storia Generale, Osservazioni fisiche,
  Raccomandazioni, Farmaci consigliati, Uso di farmaci, etc.)
- Aggiunte subsection Allergie e Terapia farmacologica in atto
  nella sezione Storia Clinica
- CT25: aggiunti entryRelationship specifici (Decorso Clinico, Stato,
  Età diagnosi patologia, reazione allergica MFST/REFR)

Risultati: 2 OK (201) + 11 KO + 10 N/A + 1 timeout
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111#MEDILUSTSRLXX/Medilust_Srl/Mami/1.0.0/report-checklist.xlsx
+++ b/GATEWAY/A1#111#MEDILUSTSRLXX/Medilust_Srl/Mami/1.0.0/report-checklist.xlsx
@@ -2932,17 +2932,17 @@
       </c>
       <c r="F15" s="31" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="G15" s="31" t="inlineStr">
         <is>
-          <t>2026-03-30T10:18:56.373142Z</t>
+          <t>2026-03-31T10:33:33.923806Z</t>
         </is>
       </c>
       <c r="H15" s="31" t="inlineStr">
         <is>
-          <t>e341915c6d3e1f472d97cdcb971fb5a2</t>
+          <t>7e529e275edcd8d2ee34c49ed654544e</t>
         </is>
       </c>
       <c r="I15" s="36" t="inlineStr">
@@ -3388,17 +3388,17 @@
       </c>
       <c r="F23" s="31" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="G23" s="31" t="inlineStr">
         <is>
-          <t>2026-03-30T10:18:56.373144Z</t>
+          <t>2026-03-31T10:33:33.923808Z</t>
         </is>
       </c>
       <c r="H23" s="31" t="inlineStr">
         <is>
-          <t>758af7b4f290de78f71ef2edaca93bed</t>
+          <t>fecbf3eb9ff591c485111d6d62b08f93</t>
         </is>
       </c>
       <c r="I23" s="36" t="inlineStr">
@@ -7973,22 +7973,22 @@
       </c>
       <c r="F116" s="31" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="G116" s="31" t="inlineStr">
         <is>
-          <t>2026-03-30T10:18:56.373146Z</t>
+          <t>2026-03-31T10:33:33.923810Z</t>
         </is>
       </c>
       <c r="H116" s="31" t="inlineStr">
         <is>
-          <t>97be6698fb0ab4b731c208d1619ce938</t>
+          <t>96fe23d6b95c41f20a5638e2bbf4b1ce</t>
         </is>
       </c>
       <c r="I116" s="36" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.331939b21588d65462217c807dfe9db215db18fd1bee3182c0582922187c37af.5cc0a65362^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.978532ae52b4dc915e3ac919fb73d48f99aef5ceb942f0438ac2b608f85d232f.66d000ad9a^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J116" s="32" t="inlineStr">
@@ -8069,22 +8069,22 @@
       </c>
       <c r="F117" s="31" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="G117" s="31" t="inlineStr">
         <is>
-          <t>2026-03-30T10:18:56.373148Z</t>
+          <t>2026-03-31T10:33:33.923812Z</t>
         </is>
       </c>
       <c r="H117" s="31" t="inlineStr">
         <is>
-          <t>9b20623b5aa59e39557174ec4bb95dff</t>
+          <t>d7275002d0ad835ee2a736604360750c</t>
         </is>
       </c>
       <c r="I117" s="36" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.11c6b0631b8cffdbe0c4dd5103ab1f3d0964fbcdd7c603d3d723f0cc0c0e9022.91e8aaf702^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.ca8802d6d6e54d965594ea683db01904dde2b4bc0b1a3199a4b8a9fc8e35f9f3.9ed07f857a^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J117" s="32" t="inlineStr">
@@ -8165,22 +8165,22 @@
       </c>
       <c r="F118" s="31" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="G118" s="31" t="inlineStr">
         <is>
-          <t>2026-03-30T10:18:56.373149Z</t>
+          <t>2026-03-31T10:33:33.923814Z</t>
         </is>
       </c>
       <c r="H118" s="31" t="inlineStr">
         <is>
-          <t>116178cc142dba50b6187bac9116c45d</t>
+          <t>b9c762e18d83a689c78fae6a2a27fc29</t>
         </is>
       </c>
       <c r="I118" s="36" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.cdc96161f479cbfa78953c74a2f82337d728fd81c8bd8b56031d7b5fb490cc12.8f6f5a8e55^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.b89f7e00ecfffef326a9ef2d5f52b6cedff5d5ef772c19de50a79342f9cdd78d.b0160be0d1^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J118" s="32" t="inlineStr">
@@ -8261,22 +8261,22 @@
       </c>
       <c r="F119" s="31" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="G119" s="31" t="inlineStr">
         <is>
-          <t>2026-03-30T10:18:56.373177Z</t>
+          <t>2026-03-31T10:33:33.923816Z</t>
         </is>
       </c>
       <c r="H119" s="31" t="inlineStr">
         <is>
-          <t>fe4f7521a2952d9f29324cc05b356501</t>
+          <t>9befc977333ed86f81e1dc82d041b15b</t>
         </is>
       </c>
       <c r="I119" s="36" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.1297897c909cfa42597c8da00d9624f362ab88b022d6a5fb9cd035204403a5f3.8802b8b879^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.bb4c71fea28045735cce69256804fbffe97181f2d4f1c5f11562468769f4ae04.dc3aade8fb^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J119" s="32" t="inlineStr">
@@ -8413,22 +8413,22 @@
       </c>
       <c r="F121" s="31" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="G121" s="31" t="inlineStr">
         <is>
-          <t>2026-03-30T10:18:56.373179Z</t>
+          <t>2026-03-31T10:33:33.923818Z</t>
         </is>
       </c>
       <c r="H121" s="31" t="inlineStr">
         <is>
-          <t>23a84357d775dff55faffa09a2c3a8c1</t>
+          <t>7e94b151a16bfda59fc187cec1b7507c</t>
         </is>
       </c>
       <c r="I121" s="36" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.71e65b5a57b9a5a687feeb43a6d8453b4f6873e7f0ecb88ba80056f9662cdec7.10080fc657^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.dd1c8c4a39ceb0ef812b0c4e5d8c46256ad99fb5e9c4265dc07f974e440c0d4d.e475bdb714^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J121" s="32" t="inlineStr">
@@ -8509,22 +8509,22 @@
       </c>
       <c r="F122" s="31" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="G122" s="31" t="inlineStr">
         <is>
-          <t>2026-03-30T10:18:56.373181Z</t>
+          <t>2026-03-31T10:33:33.923820Z</t>
         </is>
       </c>
       <c r="H122" s="31" t="inlineStr">
         <is>
-          <t>b3ce02f5258c0fb07e69fba2308ae8ef</t>
+          <t>ed9603bbebf11e02d84fa57d988b2aff</t>
         </is>
       </c>
       <c r="I122" s="36" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.3ab867b2426a85d90cc1abb1ee4408c0ee918497ed6ef337eac621bd7a161ba0.e1020f6630^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.61db9fb4873623a2a5ef237514e1d56eae017858a085ac50df30d80e2cee9f67.a8eadf7bb2^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J122" s="32" t="inlineStr">
@@ -8661,22 +8661,22 @@
       </c>
       <c r="F124" s="31" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="G124" s="31" t="inlineStr">
         <is>
-          <t>2026-03-30T10:18:56.373183Z</t>
+          <t>2026-03-31T10:33:33.923821Z</t>
         </is>
       </c>
       <c r="H124" s="31" t="inlineStr">
         <is>
-          <t>c9bd14a0ff9b7cce8e420c35b029ab58</t>
+          <t>02b169203b61f375a52e7bdb002e1b25</t>
         </is>
       </c>
       <c r="I124" s="36" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.5038033db023b45100e24712fa5fe39719c64c2479ffb28b8276ec299bea83df.7c159f6684^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.e6b4def295f1c7c0250257f69d80dd211be0293037a0dd75e817f6f01afe1fc7.fca0811adb^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J124" s="32" t="inlineStr">
@@ -9037,22 +9037,22 @@
       </c>
       <c r="F130" s="31" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="G130" s="31" t="inlineStr">
         <is>
-          <t>2026-03-30T10:18:56.373184Z</t>
+          <t>2026-03-31T10:33:33.923823Z</t>
         </is>
       </c>
       <c r="H130" s="31" t="inlineStr">
         <is>
-          <t>320a998aa085823859222a2259b4b77c</t>
+          <t>20c59eaba299b9805c58d9c26f03a2af</t>
         </is>
       </c>
       <c r="I130" s="36" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.9d8d599dbab4551922a7ec336437cd8ecf96f436900ba77e4ef6e2df3c65ec42.925f211a3d^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.55135f683adefbf94bc319c6a9d190d69da6371e38de92a02529bbcf6f3864d6.ce292a0ee8^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J130" s="32" t="inlineStr">
@@ -10731,22 +10731,22 @@
       </c>
       <c r="F164" s="31" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="G164" s="31" t="inlineStr">
         <is>
-          <t>2026-03-30T10:18:56.373085Z</t>
+          <t>2026-03-31T10:33:33.923772Z</t>
         </is>
       </c>
       <c r="H164" s="31" t="inlineStr">
         <is>
-          <t>59dc7268b603f5006cb23c0378f5eed5</t>
+          <t>198a21af55d63648384b66c6f4074a5a</t>
         </is>
       </c>
       <c r="I164" s="36" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.0dd4f3a86924a9544353276f9c0ecc9f445c9734bdbade991fcad6ecd2a60bd1.2017f9aa77^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.0913a5d3e4f754dda36be3c3d1f3dbf552254af7fc62e6180a18e985c2151379.5465a39f44^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J164" s="32" t="inlineStr">
@@ -10799,22 +10799,22 @@
       </c>
       <c r="F165" s="31" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="G165" s="31" t="inlineStr">
         <is>
-          <t>2026-03-30T10:18:56.373139Z</t>
+          <t>2026-03-31T10:33:33.923804Z</t>
         </is>
       </c>
       <c r="H165" s="31" t="inlineStr">
         <is>
-          <t>f8396c60246beea23fae8f43329dae1d</t>
+          <t>77b7aa3e9051da883fdc6adc4c9341ff</t>
         </is>
       </c>
       <c r="I165" s="36" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.f813144e0cd96b8b6652e522b89c2a5ff9c4798c6395231cce22008ea2fc958f.ca6285e102^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.f7902298d112be06492beb7c0b60351dde5e6361be42ddd6ccb5fb0dc70123a7.0ebbd90c6b^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J165" s="32" t="inlineStr">
@@ -11692,22 +11692,22 @@
       </c>
       <c r="F183" s="29" t="inlineStr">
         <is>
-          <t>2026-03-30</t>
+          <t>2026-03-31</t>
         </is>
       </c>
       <c r="G183" s="29" t="inlineStr">
         <is>
-          <t>2026-03-30T10:18:56.373186Z</t>
+          <t>2026-03-31T10:33:33.923825Z</t>
         </is>
       </c>
       <c r="H183" s="29" t="inlineStr">
         <is>
-          <t>30809de819f2718028776d2f225576f3</t>
+          <t>9c43283ab3e1ba3a709b00a6c877859e</t>
         </is>
       </c>
       <c r="I183" s="29" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.5c9418f0aee8bfae73f29e4db028b29cdca87ac640dc005a3e47fae91a89ef1c.731f7692ac^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.a82c35c3b9edd0d83652fb06572ece2a849934e8819f2b7661e7f714edbfa9cd.c9671b3fc5^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J183" s="32" t="inlineStr">

</xml_diff>

<commit_message>
Fix test 448, 449 per medilust_srl/mami/1.0.0
Aggiunta entry/observation con moodCode=EVN nella sezione
Precedenti Esami Eseguiti (ultimo errore segnalato).

CDA completo allineato ai riferimenti CT24/CT25.
Risultati: 2 OK (201) + 11 KO + 10 N/A + 1 timeout
</commit_message>
<xml_diff>
--- a/GATEWAY/A1#111#MEDILUSTSRLXX/Medilust_Srl/Mami/1.0.0/report-checklist.xlsx
+++ b/GATEWAY/A1#111#MEDILUSTSRLXX/Medilust_Srl/Mami/1.0.0/report-checklist.xlsx
@@ -2932,17 +2932,17 @@
       </c>
       <c r="F15" s="31" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="G15" s="31" t="inlineStr">
         <is>
-          <t>2026-03-31T10:33:33.923806Z</t>
+          <t>2026-04-01T05:34:40.092481Z</t>
         </is>
       </c>
       <c r="H15" s="31" t="inlineStr">
         <is>
-          <t>7e529e275edcd8d2ee34c49ed654544e</t>
+          <t>52a94cef26280a6a063d304afe7540b5</t>
         </is>
       </c>
       <c r="I15" s="36" t="inlineStr">
@@ -3388,17 +3388,17 @@
       </c>
       <c r="F23" s="31" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="G23" s="31" t="inlineStr">
         <is>
-          <t>2026-03-31T10:33:33.923808Z</t>
+          <t>2026-04-01T05:34:40.092483Z</t>
         </is>
       </c>
       <c r="H23" s="31" t="inlineStr">
         <is>
-          <t>fecbf3eb9ff591c485111d6d62b08f93</t>
+          <t>587f3b84e8622e9c38581ffe0946568c</t>
         </is>
       </c>
       <c r="I23" s="36" t="inlineStr">
@@ -7973,22 +7973,22 @@
       </c>
       <c r="F116" s="31" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="G116" s="31" t="inlineStr">
         <is>
-          <t>2026-03-31T10:33:33.923810Z</t>
+          <t>2026-04-01T05:34:40.092485Z</t>
         </is>
       </c>
       <c r="H116" s="31" t="inlineStr">
         <is>
-          <t>96fe23d6b95c41f20a5638e2bbf4b1ce</t>
+          <t>f05fd61c7c3154bd3419992db769f551</t>
         </is>
       </c>
       <c r="I116" s="36" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.978532ae52b4dc915e3ac919fb73d48f99aef5ceb942f0438ac2b608f85d232f.66d000ad9a^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.231c12f072c505811ea8a12ba89b670fe67436c530adc95a776258805a6b08c1.4711c30dab^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J116" s="32" t="inlineStr">
@@ -8069,22 +8069,22 @@
       </c>
       <c r="F117" s="31" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="G117" s="31" t="inlineStr">
         <is>
-          <t>2026-03-31T10:33:33.923812Z</t>
+          <t>2026-04-01T05:34:40.092487Z</t>
         </is>
       </c>
       <c r="H117" s="31" t="inlineStr">
         <is>
-          <t>d7275002d0ad835ee2a736604360750c</t>
+          <t>319ab7d94a201f57c871324e7fe23e7c</t>
         </is>
       </c>
       <c r="I117" s="36" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.ca8802d6d6e54d965594ea683db01904dde2b4bc0b1a3199a4b8a9fc8e35f9f3.9ed07f857a^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.4be3d7a5ee009fe184aa3e4d16ec35bb26e36e7ae59c943b1eca5806512ec07c.da9e98b3ac^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J117" s="32" t="inlineStr">
@@ -8165,22 +8165,22 @@
       </c>
       <c r="F118" s="31" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="G118" s="31" t="inlineStr">
         <is>
-          <t>2026-03-31T10:33:33.923814Z</t>
+          <t>2026-04-01T05:34:40.092614Z</t>
         </is>
       </c>
       <c r="H118" s="31" t="inlineStr">
         <is>
-          <t>b9c762e18d83a689c78fae6a2a27fc29</t>
+          <t>a7a880c153a598b70df4a4f88279cad4</t>
         </is>
       </c>
       <c r="I118" s="36" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.b89f7e00ecfffef326a9ef2d5f52b6cedff5d5ef772c19de50a79342f9cdd78d.b0160be0d1^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.4ff247ad9b0de8f727b92cc391768d4126bbaf8e98cf7a201bf7701cb755674e.861d852c78^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J118" s="32" t="inlineStr">
@@ -8261,22 +8261,22 @@
       </c>
       <c r="F119" s="31" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="G119" s="31" t="inlineStr">
         <is>
-          <t>2026-03-31T10:33:33.923816Z</t>
+          <t>2026-04-01T05:34:40.092618Z</t>
         </is>
       </c>
       <c r="H119" s="31" t="inlineStr">
         <is>
-          <t>9befc977333ed86f81e1dc82d041b15b</t>
+          <t>79a7a8fd25a1dc888bb903983850bc18</t>
         </is>
       </c>
       <c r="I119" s="36" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.bb4c71fea28045735cce69256804fbffe97181f2d4f1c5f11562468769f4ae04.dc3aade8fb^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.593459dfd444eb07a04f14292ee8ed6e371d6ff35c9ffda9c1367f2296c0c8bb.06c7d441f7^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J119" s="32" t="inlineStr">
@@ -8413,22 +8413,22 @@
       </c>
       <c r="F121" s="31" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="G121" s="31" t="inlineStr">
         <is>
-          <t>2026-03-31T10:33:33.923818Z</t>
+          <t>2026-04-01T05:34:40.092620Z</t>
         </is>
       </c>
       <c r="H121" s="31" t="inlineStr">
         <is>
-          <t>7e94b151a16bfda59fc187cec1b7507c</t>
+          <t>2249c6f8561ffac24629d8f1e4d71400</t>
         </is>
       </c>
       <c r="I121" s="36" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.dd1c8c4a39ceb0ef812b0c4e5d8c46256ad99fb5e9c4265dc07f974e440c0d4d.e475bdb714^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.bb788dd47a4efa327d96b3455cf568bde370eba60ef7bfcf59e26816c7486fb3.7684de3fb8^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J121" s="32" t="inlineStr">
@@ -8509,22 +8509,22 @@
       </c>
       <c r="F122" s="31" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="G122" s="31" t="inlineStr">
         <is>
-          <t>2026-03-31T10:33:33.923820Z</t>
+          <t>2026-04-01T05:34:40.092622Z</t>
         </is>
       </c>
       <c r="H122" s="31" t="inlineStr">
         <is>
-          <t>ed9603bbebf11e02d84fa57d988b2aff</t>
+          <t>f97b14d42920266c70872d47782d8b54</t>
         </is>
       </c>
       <c r="I122" s="36" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.61db9fb4873623a2a5ef237514e1d56eae017858a085ac50df30d80e2cee9f67.a8eadf7bb2^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.4c23cc205e2d51fc80c4b0c48dfc79fad7297e84df51013a9ec291fc35648668.c695122fd2^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J122" s="32" t="inlineStr">
@@ -8661,22 +8661,22 @@
       </c>
       <c r="F124" s="31" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="G124" s="31" t="inlineStr">
         <is>
-          <t>2026-03-31T10:33:33.923821Z</t>
+          <t>2026-04-01T05:34:40.092624Z</t>
         </is>
       </c>
       <c r="H124" s="31" t="inlineStr">
         <is>
-          <t>02b169203b61f375a52e7bdb002e1b25</t>
+          <t>e8f61d8e7c2f337b9e17081edf507ef2</t>
         </is>
       </c>
       <c r="I124" s="36" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.e6b4def295f1c7c0250257f69d80dd211be0293037a0dd75e817f6f01afe1fc7.fca0811adb^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.a652e4e022d05f751de418b905fd2edd726a9e851fa5909742cd94d40a062717.bc863b2cf2^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J124" s="32" t="inlineStr">
@@ -9037,22 +9037,22 @@
       </c>
       <c r="F130" s="31" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="G130" s="31" t="inlineStr">
         <is>
-          <t>2026-03-31T10:33:33.923823Z</t>
+          <t>2026-04-01T05:34:40.092625Z</t>
         </is>
       </c>
       <c r="H130" s="31" t="inlineStr">
         <is>
-          <t>20c59eaba299b9805c58d9c26f03a2af</t>
+          <t>593e3090c7510b3ee812cb4c3db71a71</t>
         </is>
       </c>
       <c r="I130" s="36" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.55135f683adefbf94bc319c6a9d190d69da6371e38de92a02529bbcf6f3864d6.ce292a0ee8^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.38026d2e66599e17edc8a8970cabb6cb1c005fc917063d40ba5f98bffea8f374.f122972479^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J130" s="32" t="inlineStr">
@@ -10731,22 +10731,22 @@
       </c>
       <c r="F164" s="31" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="G164" s="31" t="inlineStr">
         <is>
-          <t>2026-03-31T10:33:33.923772Z</t>
+          <t>2026-04-01T05:34:40.092355Z</t>
         </is>
       </c>
       <c r="H164" s="31" t="inlineStr">
         <is>
-          <t>198a21af55d63648384b66c6f4074a5a</t>
+          <t>e744ab721dda8bd1e806880ee5259775</t>
         </is>
       </c>
       <c r="I164" s="36" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.0913a5d3e4f754dda36be3c3d1f3dbf552254af7fc62e6180a18e985c2151379.5465a39f44^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.80a60ac3b7a0f9cb4e954a0ed719c7aaadc1b25419732ac82d34f1440c19ce09.a3811df9c1^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J164" s="32" t="inlineStr">
@@ -10799,22 +10799,22 @@
       </c>
       <c r="F165" s="31" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="G165" s="31" t="inlineStr">
         <is>
-          <t>2026-03-31T10:33:33.923804Z</t>
+          <t>2026-04-01T05:34:40.092478Z</t>
         </is>
       </c>
       <c r="H165" s="31" t="inlineStr">
         <is>
-          <t>77b7aa3e9051da883fdc6adc4c9341ff</t>
+          <t>855837d7039569c5b5e39ec12f2534d2</t>
         </is>
       </c>
       <c r="I165" s="36" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.f7902298d112be06492beb7c0b60351dde5e6361be42ddd6ccb5fb0dc70123a7.0ebbd90c6b^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.c755b909346fcc217cb14b935084a74217ffa89b396120a193cadb13211e1261.cadc5e8231^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J165" s="32" t="inlineStr">
@@ -11692,22 +11692,22 @@
       </c>
       <c r="F183" s="29" t="inlineStr">
         <is>
-          <t>2026-03-31</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="G183" s="29" t="inlineStr">
         <is>
-          <t>2026-03-31T10:33:33.923825Z</t>
+          <t>2026-04-01T05:34:40.092627Z</t>
         </is>
       </c>
       <c r="H183" s="29" t="inlineStr">
         <is>
-          <t>9c43283ab3e1ba3a709b00a6c877859e</t>
+          <t>ec57ed4c0ee3d18a10ddbfa138d354be</t>
         </is>
       </c>
       <c r="I183" s="29" t="inlineStr">
         <is>
-          <t>2.16.840.1.113883.2.9.2.120.4.4.a82c35c3b9edd0d83652fb06572ece2a849934e8819f2b7661e7f714edbfa9cd.c9671b3fc5^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
+          <t>2.16.840.1.113883.2.9.2.120.4.4.791165104c5b196acd6e5eec8b9fd73780ad2e499bc67325dc47b617b1be7e28.58f45f2c70^^^^urn:ihe:iti:xdw:2013:workflowInstanceId</t>
         </is>
       </c>
       <c r="J183" s="32" t="inlineStr">

</xml_diff>